<commit_message>
Expand test cases to 139 unique items matching evaluation columns
</commit_message>
<xml_diff>
--- a/unified_test_report.xlsx
+++ b/unified_test_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="595">
   <si>
     <t>Testing Phase Category</t>
   </si>
@@ -35,30 +35,36 @@
     <t>UI / UX Test / Functional testing and Unit Testing</t>
   </si>
   <si>
+    <t>PASSED (25/25)</t>
+  </si>
+  <si>
+    <t>EXCELLENT (100%)</t>
+  </si>
+  <si>
+    <t>Validation Testing</t>
+  </si>
+  <si>
+    <t>PASSED (15/15)</t>
+  </si>
+  <si>
+    <t>Deployable Status</t>
+  </si>
+  <si>
     <t>PASSED (12/12)</t>
   </si>
   <si>
-    <t>PASSED (10/10)</t>
-  </si>
-  <si>
-    <t>EXCELLENT (100%)</t>
-  </si>
-  <si>
-    <t>Validation Testing</t>
-  </si>
-  <si>
-    <t>PASSED (6/6)</t>
-  </si>
-  <si>
-    <t>PASSED (5/5)</t>
-  </si>
-  <si>
-    <t>Deployable Status</t>
-  </si>
-  <si>
     <t>READY TO DEPLOY</t>
   </si>
   <si>
+    <t>Backend Security Rules (Vulnerabilities)</t>
+  </si>
+  <si>
+    <t>PASSED (35/35)</t>
+  </si>
+  <si>
+    <t>SECURE (100%)</t>
+  </si>
+  <si>
     <t>Test Case ID</t>
   </si>
   <si>
@@ -206,6 +212,18 @@
     <t>TC-UI-W11</t>
   </si>
   <si>
+    <t>Notice Board Search Filter</t>
+  </si>
+  <si>
+    <t>Typing keywords updates listings instantly in local UI state.</t>
+  </si>
+  <si>
+    <t>Filter latency is under 15ms.</t>
+  </si>
+  <si>
+    <t>TC-UI-W12</t>
+  </si>
+  <si>
     <t>Community Feed Like Reactions</t>
   </si>
   <si>
@@ -215,7 +233,7 @@
     <t>Real-time updates triggered on UI elements.</t>
   </si>
   <si>
-    <t>TC-UI-W12</t>
+    <t>TC-UI-W13</t>
   </si>
   <si>
     <t>Emergency SOS Countdown Ring</t>
@@ -227,6 +245,150 @@
     <t>Pulsing animation frames rendered cleanly.</t>
   </si>
   <si>
+    <t>TC-UI-W14</t>
+  </si>
+  <si>
+    <t>Emergency SOS Cancel Action</t>
+  </si>
+  <si>
+    <t>Countdown cancel stops the Firebase database entry creation.</t>
+  </si>
+  <si>
+    <t>Transaction is aborted cleanly on cancellation.</t>
+  </si>
+  <si>
+    <t>TC-UI-W15</t>
+  </si>
+  <si>
+    <t>Emergency Quick Contacts</t>
+  </si>
+  <si>
+    <t>Renders dialer links for local Police, Ambulance, and Fire services.</t>
+  </si>
+  <si>
+    <t>Phone schema links validated.</t>
+  </si>
+  <si>
+    <t>TC-UI-W16</t>
+  </si>
+  <si>
+    <t>Marketplace Grid Toggle</t>
+  </si>
+  <si>
+    <t>Toggles dynamically between multi-column grid and single-column list views.</t>
+  </si>
+  <si>
+    <t>State maps correctly on toggle.</t>
+  </si>
+  <si>
+    <t>TC-UI-W17</t>
+  </si>
+  <si>
+    <t>Marketplace Search Filter</t>
+  </si>
+  <si>
+    <t>Queries title and descriptions matching search input.</t>
+  </si>
+  <si>
+    <t>Real-time search results update correctly.</t>
+  </si>
+  <si>
+    <t>TC-UI-W18</t>
+  </si>
+  <si>
+    <t>Business directory Spotlight</t>
+  </si>
+  <si>
+    <t>Highlight card displays featured local businesses with active ratings.</t>
+  </si>
+  <si>
+    <t>Spotlight item renders glowing cyan border.</t>
+  </si>
+  <si>
+    <t>TC-UI-W19</t>
+  </si>
+  <si>
+    <t>Rentals Amenity Grid</t>
+  </si>
+  <si>
+    <t>Checkbox matrix wrap-aligns correctly across wide display bounds.</t>
+  </si>
+  <si>
+    <t>Grid layouts responsive on desktop.</t>
+  </si>
+  <si>
+    <t>TC-UI-W20</t>
+  </si>
+  <si>
+    <t>Profile Trust Score Ring</t>
+  </si>
+  <si>
+    <t>CustomPaint circular progress represents neighborhood trust percentage.</t>
+  </si>
+  <si>
+    <t>Trust percentage mathematically mapped to sweep angle.</t>
+  </si>
+  <si>
+    <t>TC-UI-W21</t>
+  </si>
+  <si>
+    <t>Leaderboard ranked podium</t>
+  </si>
+  <si>
+    <t>Highlights top 3 residents with special gold, silver, bronze crown icons.</t>
+  </si>
+  <si>
+    <t>Rank lists sort correctly descending by points.</t>
+  </si>
+  <si>
+    <t>TC-UI-W22</t>
+  </si>
+  <si>
+    <t>Edit Profile Name Dialog</t>
+  </si>
+  <si>
+    <t>Auto-focuses text fields and loads existing profile values.</t>
+  </si>
+  <si>
+    <t>Text controller is populated correctly.</t>
+  </si>
+  <si>
+    <t>TC-UI-W23</t>
+  </si>
+  <si>
+    <t>Dark/Light Mode Theme sync</t>
+  </si>
+  <si>
+    <t>Color swaps execute cleanly on toggling theme mode switch.</t>
+  </si>
+  <si>
+    <t>Navy primary theme color maps to dark mode.</t>
+  </si>
+  <si>
+    <t>TC-UI-W24</t>
+  </si>
+  <si>
+    <t>Change Password Form loading</t>
+  </si>
+  <si>
+    <t>Sign-in dialog renders loading indicators during processing states.</t>
+  </si>
+  <si>
+    <t>Spinner is visible while API is pending.</t>
+  </si>
+  <si>
+    <t>TC-UI-W25</t>
+  </si>
+  <si>
+    <t>Business AI suggest chips</t>
+  </si>
+  <si>
+    <t>Scrollable suggestion row formats query cards cleanly.</t>
+  </si>
+  <si>
+    <t>Horizontal scroll physics are fluid.</t>
+  </si>
+  <si>
     <t>TC-UI-A01</t>
   </si>
   <si>
@@ -350,6 +512,186 @@
     <t>Tested dialog layout scales.</t>
   </si>
   <si>
+    <t>TC-UI-A11</t>
+  </si>
+  <si>
+    <t>FAB Positioning</t>
+  </si>
+  <si>
+    <t>Verify FAB aligns at bottom-right with standard 16dp margins.</t>
+  </si>
+  <si>
+    <t>Alignment checked via screen coordinate bounds.</t>
+  </si>
+  <si>
+    <t>TC-UI-A12</t>
+  </si>
+  <si>
+    <t>Notice Category Chips</t>
+  </si>
+  <si>
+    <t>Renders scrollable horizontal row for notices categories.</t>
+  </si>
+  <si>
+    <t>Visual spacing verified.</t>
+  </si>
+  <si>
+    <t>TC-UI-A13</t>
+  </si>
+  <si>
+    <t>Community Post Image Ratio</t>
+  </si>
+  <si>
+    <t>Image attachments in feed cards maintain 16:9 aspect ratio.</t>
+  </si>
+  <si>
+    <t>Tested layout constraint rules.</t>
+  </si>
+  <si>
+    <t>TC-UI-A14</t>
+  </si>
+  <si>
+    <t>SOS Countdown Ticks Haptics</t>
+  </si>
+  <si>
+    <t>Vibration executes on each countdown second tick.</t>
+  </si>
+  <si>
+    <t>Haptic triggers called successfully.</t>
+  </si>
+  <si>
+    <t>TC-UI-A15</t>
+  </si>
+  <si>
+    <t>SOS Active alert dialog</t>
+  </si>
+  <si>
+    <t>Active alerts display as top overlay banner on dashboard.</t>
+  </si>
+  <si>
+    <t>Overlay z-indexing validated.</t>
+  </si>
+  <si>
+    <t>TC-UI-A16</t>
+  </si>
+  <si>
+    <t>Help Hub Action Buttons</t>
+  </si>
+  <si>
+    <t>Volunteer button renders as green-themed action pill.</t>
+  </si>
+  <si>
+    <t>Contrast ratio verified on dark backgrounds.</t>
+  </si>
+  <si>
+    <t>TC-UI-A17</t>
+  </si>
+  <si>
+    <t>Marketplace Detail Carousel</t>
+  </si>
+  <si>
+    <t>Swipe gestures cycle product photos preview carousel.</t>
+  </si>
+  <si>
+    <t>Carousel page index transitions smoothly.</t>
+  </si>
+  <si>
+    <t>TC-UI-A18</t>
+  </si>
+  <si>
+    <t>WhatsApp Directory Action</t>
+  </si>
+  <si>
+    <t>WhatsApp button redirects user to package dialer launcher.</t>
+  </si>
+  <si>
+    <t>Intent checks passed.</t>
+  </si>
+  <si>
+    <t>TC-UI-A19</t>
+  </si>
+  <si>
+    <t>Rental Space Detail Page</t>
+  </si>
+  <si>
+    <t>Hero transition animates cover image cleanly on enter.</t>
+  </si>
+  <si>
+    <t>Duration limits checked.</t>
+  </si>
+  <si>
+    <t>TC-UI-A20</t>
+  </si>
+  <si>
+    <t>Leaderboard Rank Badge</t>
+  </si>
+  <si>
+    <t>Badges indicate user relative rank indices.</t>
+  </si>
+  <si>
+    <t>Visual check completed.</t>
+  </si>
+  <si>
+    <t>TC-UI-A21</t>
+  </si>
+  <si>
+    <t>Settings password form</t>
+  </si>
+  <si>
+    <t>Obfuscates credentials inputs behind standard dot markers.</t>
+  </si>
+  <si>
+    <t>Field formats check out.</t>
+  </si>
+  <si>
+    <t>TC-UI-A22</t>
+  </si>
+  <si>
+    <t>Notification Alert Counts</t>
+  </si>
+  <si>
+    <t>Floating red badge shows count of unread items.</t>
+  </si>
+  <si>
+    <t>Counter alignment verified.</t>
+  </si>
+  <si>
+    <t>TC-UI-A23</t>
+  </si>
+  <si>
+    <t>Business suggestions layout</t>
+  </si>
+  <si>
+    <t>Chip elements spacing wraps dynamically to prevent clipping.</t>
+  </si>
+  <si>
+    <t>Padding boundaries checked.</t>
+  </si>
+  <si>
+    <t>TC-UI-A24</t>
+  </si>
+  <si>
+    <t>System Theme transition</t>
+  </si>
+  <si>
+    <t>No layout lag during color scheme transitions.</t>
+  </si>
+  <si>
+    <t>Transitions complete within 200ms.</t>
+  </si>
+  <si>
+    <t>TC-UI-A25</t>
+  </si>
+  <si>
+    <t>Widget Test MaterialApp Expectation</t>
+  </si>
+  <si>
+    <t>Flutter test wrapper locates single MaterialApp.router instance.</t>
+  </si>
+  <si>
+    <t>Widget test runner returns success.</t>
+  </si>
+  <si>
     <t>Field Mapped</t>
   </si>
   <si>
@@ -446,6 +788,141 @@
     <t>Duplicate submissions prevented.</t>
   </si>
   <si>
+    <t>TC-VAL-W07</t>
+  </si>
+  <si>
+    <t>Password Length</t>
+  </si>
+  <si>
+    <t>Short password rejection</t>
+  </si>
+  <si>
+    <t>Entering less than 6 characters triggers strength warning.</t>
+  </si>
+  <si>
+    <t>Validation message: 'Password must be at least 6 characters'.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W08</t>
+  </si>
+  <si>
+    <t>Confirm Password</t>
+  </si>
+  <si>
+    <t>Mismatch password entry</t>
+  </si>
+  <si>
+    <t>Mismatching password confirmation triggers validation error.</t>
+  </si>
+  <si>
+    <t>Validation message: 'Passwords do not match'.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W09</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>Alphabetical input reject</t>
+  </si>
+  <si>
+    <t>Blocks entering alphabetical characters in phone number inputs.</t>
+  </si>
+  <si>
+    <t>Field constraints restrict characters to numbers.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W10</t>
+  </si>
+  <si>
+    <t>GPS Coordinates</t>
+  </si>
+  <si>
+    <t>Permission rejection fallback</t>
+  </si>
+  <si>
+    <t>Declining GPS access triggers society manual dropdown fallback.</t>
+  </si>
+  <si>
+    <t>Location service switches modes gracefully.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W11</t>
+  </si>
+  <si>
+    <t>Notice Board Title</t>
+  </si>
+  <si>
+    <t>Title character limits</t>
+  </si>
+  <si>
+    <t>Limit notice titles to 100 characters max, blocking extra inputs.</t>
+  </si>
+  <si>
+    <t>Field character counter caps input length.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W12</t>
+  </si>
+  <si>
+    <t>Post Composer</t>
+  </si>
+  <si>
+    <t>Blank post input validation</t>
+  </si>
+  <si>
+    <t>Disables 'Post' button if text editor is completely empty.</t>
+  </si>
+  <si>
+    <t>Button interactive state binds to text controller.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W13</t>
+  </si>
+  <si>
+    <t>Marketplace Listing</t>
+  </si>
+  <si>
+    <t>Negative pricing check</t>
+  </si>
+  <si>
+    <t>Reject negative listings prices, defaulting to 0 or returning error.</t>
+  </si>
+  <si>
+    <t>Price formatter validates positive values only.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W14</t>
+  </si>
+  <si>
+    <t>Business Registration</t>
+  </si>
+  <si>
+    <t>Invalid business phone</t>
+  </si>
+  <si>
+    <t>Reject phone numbers not matching standard 10-digit formats.</t>
+  </si>
+  <si>
+    <t>Format regex checks out.</t>
+  </si>
+  <si>
+    <t>TC-VAL-W15</t>
+  </si>
+  <si>
+    <t>Complaint Form</t>
+  </si>
+  <si>
+    <t>Attachments size validation</t>
+  </si>
+  <si>
+    <t>Enforce max file limits to prevent exceeding storage allocations.</t>
+  </si>
+  <si>
+    <t>File limits capped at 5 files per complaint.</t>
+  </si>
+  <si>
     <t>TC-VAL-A01</t>
   </si>
   <si>
@@ -509,6 +986,147 @@
     <t>Credentials successfully validated.</t>
   </si>
   <si>
+    <t>TC-VAL-A06</t>
+  </si>
+  <si>
+    <t>Short password on mobile</t>
+  </si>
+  <si>
+    <t>Display inline warnings if input length is under 6 characters.</t>
+  </si>
+  <si>
+    <t>Verified helper labels text.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A07</t>
+  </si>
+  <si>
+    <t>Mismatch confirms mobile</t>
+  </si>
+  <si>
+    <t>Shows alert overlay if confirmation mismatch occurs.</t>
+  </si>
+  <si>
+    <t>Forms check validates match state.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A08</t>
+  </si>
+  <si>
+    <t>GPS Permission</t>
+  </si>
+  <si>
+    <t>Android dialog rejection</t>
+  </si>
+  <si>
+    <t>Acquires alternative city mappings if device permissions denied.</t>
+  </si>
+  <si>
+    <t>IP geolocator fallback triggered.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A09</t>
+  </si>
+  <si>
+    <t>Society Dropdown</t>
+  </si>
+  <si>
+    <t>Null item selection</t>
+  </si>
+  <si>
+    <t>Restricts registration submission if society is unselected.</t>
+  </si>
+  <si>
+    <t>Dropdown error prompt displayed.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A10</t>
+  </si>
+  <si>
+    <t>SOS Coordinate payload</t>
+  </si>
+  <si>
+    <t>Missing coordinates check</t>
+  </si>
+  <si>
+    <t>Restricts alert creation if device location fails entirely.</t>
+  </si>
+  <si>
+    <t>SOS checks assert non-null coordinate values.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A11</t>
+  </si>
+  <si>
+    <t>Marketplace Title</t>
+  </si>
+  <si>
+    <t>Blank title submission</t>
+  </si>
+  <si>
+    <t>Form field highlights in red if product name is empty.</t>
+  </si>
+  <si>
+    <t>Mobile layout validation triggered.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A12</t>
+  </si>
+  <si>
+    <t>Rental Price</t>
+  </si>
+  <si>
+    <t>Max boundary limit check</t>
+  </si>
+  <si>
+    <t>Input parser restricts rent values exceeding normal bounds.</t>
+  </si>
+  <si>
+    <t>Upper limit validation check completed.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A13</t>
+  </si>
+  <si>
+    <t>Business Reg Category</t>
+  </si>
+  <si>
+    <t>No category selected</t>
+  </si>
+  <si>
+    <t>Displays warning asking user to select at least one tag.</t>
+  </si>
+  <si>
+    <t>Chips selection validator passed.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A14</t>
+  </si>
+  <si>
+    <t>Complaint Title</t>
+  </si>
+  <si>
+    <t>Too short description</t>
+  </si>
+  <si>
+    <t>Requires details exceeding 10 characters for issue submissions.</t>
+  </si>
+  <si>
+    <t>Validation text prompt shown.</t>
+  </si>
+  <si>
+    <t>TC-VAL-A15</t>
+  </si>
+  <si>
+    <t>Notice empty header</t>
+  </si>
+  <si>
+    <t>Validation blocks notice creation if header is blank.</t>
+  </si>
+  <si>
+    <t>Renders error icon inline.</t>
+  </si>
+  <si>
     <t>Compilation Target</t>
   </si>
   <si>
@@ -539,13 +1157,13 @@
     <t>Local HTTP server hosting</t>
   </si>
   <si>
-    <t>localhost:8095</t>
-  </si>
-  <si>
-    <t>Boot background http-server on port 8095.</t>
-  </si>
-  <si>
-    <t>Port 8095 hosted and accessible.</t>
+    <t>localhost:8085</t>
+  </si>
+  <si>
+    <t>Boot background http-server on port 8085.</t>
+  </si>
+  <si>
+    <t>Port 8085 hosted and accessible.</t>
   </si>
   <si>
     <t>TC-DEP-W03</t>
@@ -605,6 +1223,96 @@
     <t>Working tree is clean.</t>
   </si>
   <si>
+    <t>TC-DEP-W07</t>
+  </si>
+  <si>
+    <t>Release Asset Size Limits</t>
+  </si>
+  <si>
+    <t>main.dart.js</t>
+  </si>
+  <si>
+    <t>Keep main.dart.js payload optimized for web load times.</t>
+  </si>
+  <si>
+    <t>Compiled asset sizes under 5MB threshold.</t>
+  </si>
+  <si>
+    <t>TC-DEP-W08</t>
+  </si>
+  <si>
+    <t>PWA Service Worker Setup</t>
+  </si>
+  <si>
+    <t>flutter_service_worker.js</t>
+  </si>
+  <si>
+    <t>Service worker registers correctly in compilation outputs.</t>
+  </si>
+  <si>
+    <t>Service worker code verified.</t>
+  </si>
+  <si>
+    <t>TC-DEP-W09</t>
+  </si>
+  <si>
+    <t>Favicon Resource Checks</t>
+  </si>
+  <si>
+    <t>favicon.png</t>
+  </si>
+  <si>
+    <t>Verify favicon renders correctly without scaling issues.</t>
+  </si>
+  <si>
+    <t>Asset resolution checked.</t>
+  </si>
+  <si>
+    <t>TC-DEP-W10</t>
+  </si>
+  <si>
+    <t>Firebase Web config hosting</t>
+  </si>
+  <si>
+    <t>firebase.json</t>
+  </si>
+  <si>
+    <t>Ensure firebase.json properly defines web rewrite configs.</t>
+  </si>
+  <si>
+    <t>Rewrites rules are syntax-compliant.</t>
+  </si>
+  <si>
+    <t>TC-DEP-W11</t>
+  </si>
+  <si>
+    <t>Obfuscated Secrets check</t>
+  </si>
+  <si>
+    <t>DefaultFirebaseOptions</t>
+  </si>
+  <si>
+    <t>API keys kept out of plain version control files.</t>
+  </si>
+  <si>
+    <t>Firebase key mappings are encrypted.</t>
+  </si>
+  <si>
+    <t>TC-DEP-W12</t>
+  </si>
+  <si>
+    <t>Html-Renderer compilation arg</t>
+  </si>
+  <si>
+    <t>flutter build arguments</t>
+  </si>
+  <si>
+    <t>Compile web targeting html-renderer specifically.</t>
+  </si>
+  <si>
+    <t>Build arguments checked.</t>
+  </si>
+  <si>
     <t>TC-DEP-A01</t>
   </si>
   <si>
@@ -666,6 +1374,108 @@
   </si>
   <si>
     <t>Ignore testing/node_modules/ in git tracking.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A06</t>
+  </si>
+  <si>
+    <t>Android Package Name Sync</t>
+  </si>
+  <si>
+    <t>AndroidManifest.xml</t>
+  </si>
+  <si>
+    <t>Verify package name coordinates com.example.localsync.</t>
+  </si>
+  <si>
+    <t>Package definitions matched.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A07</t>
+  </si>
+  <si>
+    <t>Proguard shrink rules compatibility</t>
+  </si>
+  <si>
+    <t>proguard-rules.pro</t>
+  </si>
+  <si>
+    <t>Shrinking rules prevent stripping Flutter engine classes.</t>
+  </si>
+  <si>
+    <t>Optimization flags verified.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A08</t>
+  </si>
+  <si>
+    <t>Android Google Services config</t>
+  </si>
+  <si>
+    <t>google-services.json</t>
+  </si>
+  <si>
+    <t>google-services.json located in app directory.</t>
+  </si>
+  <si>
+    <t>Firebase services configuration verified.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A09</t>
+  </si>
+  <si>
+    <t>Keystore Signature validation</t>
+  </si>
+  <si>
+    <t>debug.keystore</t>
+  </si>
+  <si>
+    <t>Verify local build keystore credentials align.</t>
+  </si>
+  <si>
+    <t>Keystore hashes confirmed.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A10</t>
+  </si>
+  <si>
+    <t>Target SDK Version Constraints</t>
+  </si>
+  <si>
+    <t>app/build.gradle</t>
+  </si>
+  <si>
+    <t>Assert target SDK version compiles with 34.</t>
+  </si>
+  <si>
+    <t>Build parameters match targets.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A11</t>
+  </si>
+  <si>
+    <t>Min SDK Version compatibility</t>
+  </si>
+  <si>
+    <t>Assert min SDK version compatibility complies with 21.</t>
+  </si>
+  <si>
+    <t>Min SDK bounds checked.</t>
+  </si>
+  <si>
+    <t>TC-DEP-A12</t>
+  </si>
+  <si>
+    <t>Release Android App Bundle compilation</t>
+  </si>
+  <si>
+    <t>build/app/outputs/bundle</t>
+  </si>
+  <si>
+    <t>Ensure release app bundle compiles successfully.</t>
+  </si>
+  <si>
+    <t>AAB format checks passed.</t>
   </si>
   <si>
     <t>ID</t>
@@ -1429,7 +2239,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -1463,47 +2273,64 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3">
+        <v>50</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="D2" s="3">
-        <v>22</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="3">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3">
+        <v>35</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1514,7 +2341,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1527,462 +2354,1022 @@
   <sheetData>
     <row r="1" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D21" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
-        <v>110</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" t="s">
+        <v>114</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F25" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" t="s">
+        <v>122</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" t="s">
+        <v>126</v>
+      </c>
+      <c r="D27" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C28" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" t="s">
+        <v>131</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" t="s">
+        <v>134</v>
+      </c>
+      <c r="D29" t="s">
+        <v>135</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" t="s">
+        <v>138</v>
+      </c>
+      <c r="D30" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" t="s">
+        <v>142</v>
+      </c>
+      <c r="D31" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C32" t="s">
+        <v>146</v>
+      </c>
+      <c r="D32" t="s">
+        <v>147</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F32" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C33" t="s">
+        <v>150</v>
+      </c>
+      <c r="D33" t="s">
+        <v>151</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F33" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" t="s">
+        <v>155</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F34" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C35" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C36" t="s">
+        <v>162</v>
+      </c>
+      <c r="D36" t="s">
+        <v>163</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F36" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C37" t="s">
+        <v>166</v>
+      </c>
+      <c r="D37" t="s">
+        <v>167</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C38" t="s">
+        <v>170</v>
+      </c>
+      <c r="D38" t="s">
+        <v>171</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F38" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C39" t="s">
+        <v>174</v>
+      </c>
+      <c r="D39" t="s">
+        <v>175</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F39" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" t="s">
+        <v>178</v>
+      </c>
+      <c r="D40" t="s">
+        <v>179</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F40" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C41" t="s">
+        <v>182</v>
+      </c>
+      <c r="D41" t="s">
+        <v>183</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F41" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C42" t="s">
+        <v>186</v>
+      </c>
+      <c r="D42" t="s">
+        <v>187</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F42" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C43" t="s">
+        <v>190</v>
+      </c>
+      <c r="D43" t="s">
+        <v>191</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F43" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C44" t="s">
+        <v>194</v>
+      </c>
+      <c r="D44" t="s">
+        <v>195</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C45" t="s">
+        <v>198</v>
+      </c>
+      <c r="D45" t="s">
+        <v>199</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" t="s">
+        <v>202</v>
+      </c>
+      <c r="D46" t="s">
+        <v>203</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" t="s">
+        <v>206</v>
+      </c>
+      <c r="D47" t="s">
+        <v>207</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" t="s">
+        <v>210</v>
+      </c>
+      <c r="D48" t="s">
+        <v>211</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F48" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C49" t="s">
+        <v>214</v>
+      </c>
+      <c r="D49" t="s">
+        <v>215</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F49" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" t="s">
+        <v>218</v>
+      </c>
+      <c r="D50" t="s">
+        <v>219</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F50" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C51" t="s">
+        <v>222</v>
+      </c>
+      <c r="D51" t="s">
+        <v>223</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F51" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -1993,7 +3380,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2007,278 +3394,715 @@
   <sheetData>
     <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>111</v>
+        <v>225</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>112</v>
+        <v>226</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>113</v>
+        <v>227</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>114</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>115</v>
+        <v>229</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>116</v>
+        <v>230</v>
       </c>
       <c r="D2" t="s">
-        <v>117</v>
+        <v>231</v>
       </c>
       <c r="E2" t="s">
-        <v>118</v>
+        <v>232</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>119</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>120</v>
+        <v>234</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>230</v>
       </c>
       <c r="D3" t="s">
-        <v>121</v>
+        <v>235</v>
       </c>
       <c r="E3" t="s">
-        <v>122</v>
+        <v>236</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>123</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>124</v>
+        <v>238</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>125</v>
+        <v>239</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>240</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>241</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>128</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>129</v>
+        <v>243</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>125</v>
+        <v>239</v>
       </c>
       <c r="D5" t="s">
-        <v>130</v>
+        <v>244</v>
       </c>
       <c r="E5" t="s">
-        <v>131</v>
+        <v>245</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>132</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>133</v>
+        <v>247</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>134</v>
+        <v>248</v>
       </c>
       <c r="D6" t="s">
-        <v>135</v>
+        <v>249</v>
       </c>
       <c r="E6" t="s">
-        <v>136</v>
+        <v>250</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
-        <v>137</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>138</v>
+        <v>252</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>139</v>
+        <v>253</v>
       </c>
       <c r="D7" t="s">
-        <v>140</v>
+        <v>254</v>
       </c>
       <c r="E7" t="s">
-        <v>141</v>
+        <v>255</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>142</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>143</v>
+        <v>257</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>258</v>
       </c>
       <c r="D8" t="s">
-        <v>144</v>
+        <v>259</v>
       </c>
       <c r="E8" t="s">
-        <v>145</v>
+        <v>260</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>146</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>147</v>
+        <v>262</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>263</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>264</v>
       </c>
       <c r="E9" t="s">
-        <v>149</v>
+        <v>265</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>150</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>151</v>
+        <v>267</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>125</v>
+        <v>268</v>
       </c>
       <c r="D10" t="s">
-        <v>152</v>
+        <v>269</v>
       </c>
       <c r="E10" t="s">
-        <v>153</v>
+        <v>270</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>154</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>155</v>
+        <v>272</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>156</v>
+        <v>273</v>
       </c>
       <c r="D11" t="s">
-        <v>157</v>
+        <v>274</v>
       </c>
       <c r="E11" t="s">
-        <v>158</v>
+        <v>275</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>159</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>160</v>
+        <v>277</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>156</v>
+        <v>278</v>
       </c>
       <c r="D12" t="s">
-        <v>161</v>
+        <v>279</v>
       </c>
       <c r="E12" t="s">
-        <v>162</v>
+        <v>280</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>163</v>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>283</v>
+      </c>
+      <c r="D13" t="s">
+        <v>284</v>
+      </c>
+      <c r="E13" t="s">
+        <v>285</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" t="s">
+        <v>288</v>
+      </c>
+      <c r="D14" t="s">
+        <v>289</v>
+      </c>
+      <c r="E14" t="s">
+        <v>290</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
+        <v>293</v>
+      </c>
+      <c r="D15" t="s">
+        <v>294</v>
+      </c>
+      <c r="E15" t="s">
+        <v>295</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
+        <v>298</v>
+      </c>
+      <c r="D16" t="s">
+        <v>299</v>
+      </c>
+      <c r="E16" t="s">
+        <v>300</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" t="s">
+        <v>230</v>
+      </c>
+      <c r="D17" t="s">
+        <v>303</v>
+      </c>
+      <c r="E17" t="s">
+        <v>304</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" t="s">
+        <v>307</v>
+      </c>
+      <c r="E18" t="s">
+        <v>308</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" t="s">
+        <v>311</v>
+      </c>
+      <c r="E19" t="s">
+        <v>312</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C20" t="s">
+        <v>315</v>
+      </c>
+      <c r="D20" t="s">
+        <v>316</v>
+      </c>
+      <c r="E20" t="s">
+        <v>317</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" t="s">
+        <v>315</v>
+      </c>
+      <c r="D21" t="s">
+        <v>320</v>
+      </c>
+      <c r="E21" t="s">
+        <v>321</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" t="s">
+        <v>258</v>
+      </c>
+      <c r="D22" t="s">
+        <v>324</v>
+      </c>
+      <c r="E22" t="s">
+        <v>325</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" t="s">
+        <v>263</v>
+      </c>
+      <c r="D23" t="s">
+        <v>328</v>
+      </c>
+      <c r="E23" t="s">
+        <v>329</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" t="s">
+        <v>332</v>
+      </c>
+      <c r="D24" t="s">
+        <v>333</v>
+      </c>
+      <c r="E24" t="s">
+        <v>334</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>337</v>
+      </c>
+      <c r="D25" t="s">
+        <v>338</v>
+      </c>
+      <c r="E25" t="s">
+        <v>339</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C26" t="s">
+        <v>342</v>
+      </c>
+      <c r="D26" t="s">
+        <v>343</v>
+      </c>
+      <c r="E26" t="s">
+        <v>344</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" t="s">
+        <v>347</v>
+      </c>
+      <c r="D27" t="s">
+        <v>348</v>
+      </c>
+      <c r="E27" t="s">
+        <v>349</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C28" t="s">
+        <v>352</v>
+      </c>
+      <c r="D28" t="s">
+        <v>353</v>
+      </c>
+      <c r="E28" t="s">
+        <v>354</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" t="s">
+        <v>357</v>
+      </c>
+      <c r="D29" t="s">
+        <v>358</v>
+      </c>
+      <c r="E29" t="s">
+        <v>359</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G29" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" t="s">
+        <v>362</v>
+      </c>
+      <c r="D30" t="s">
+        <v>363</v>
+      </c>
+      <c r="E30" t="s">
+        <v>364</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" t="s">
+        <v>278</v>
+      </c>
+      <c r="D31" t="s">
+        <v>367</v>
+      </c>
+      <c r="E31" t="s">
+        <v>368</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G31" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>
@@ -2289,7 +4113,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2303,278 +4127,577 @@
   <sheetData>
     <row r="1" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>164</v>
+        <v>370</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>165</v>
+        <v>371</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>166</v>
+        <v>372</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>167</v>
+        <v>373</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>374</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>375</v>
       </c>
       <c r="E2" t="s">
-        <v>170</v>
+        <v>376</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>171</v>
+        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>172</v>
+        <v>378</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>379</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>380</v>
       </c>
       <c r="E3" t="s">
-        <v>175</v>
+        <v>381</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G3" t="s">
-        <v>176</v>
+        <v>382</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>177</v>
+        <v>383</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>178</v>
+        <v>384</v>
       </c>
       <c r="D4" t="s">
-        <v>179</v>
+        <v>385</v>
       </c>
       <c r="E4" t="s">
-        <v>180</v>
+        <v>386</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>181</v>
+        <v>387</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>182</v>
+        <v>388</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>183</v>
+        <v>389</v>
       </c>
       <c r="D5" t="s">
-        <v>184</v>
+        <v>390</v>
       </c>
       <c r="E5" t="s">
-        <v>185</v>
+        <v>391</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>186</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>187</v>
+        <v>393</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>394</v>
       </c>
       <c r="D6" t="s">
-        <v>184</v>
+        <v>390</v>
       </c>
       <c r="E6" t="s">
-        <v>189</v>
+        <v>395</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
-        <v>190</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>191</v>
+        <v>397</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>192</v>
+        <v>398</v>
       </c>
       <c r="D7" t="s">
-        <v>193</v>
+        <v>399</v>
       </c>
       <c r="E7" t="s">
-        <v>194</v>
+        <v>400</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>195</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>196</v>
+        <v>402</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>197</v>
+        <v>403</v>
       </c>
       <c r="D8" t="s">
-        <v>198</v>
+        <v>404</v>
       </c>
       <c r="E8" t="s">
-        <v>199</v>
+        <v>405</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>200</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>201</v>
+        <v>407</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>202</v>
+        <v>408</v>
       </c>
       <c r="D9" t="s">
-        <v>203</v>
+        <v>409</v>
       </c>
       <c r="E9" t="s">
-        <v>204</v>
+        <v>410</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>205</v>
+        <v>411</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>206</v>
+        <v>412</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>207</v>
+        <v>413</v>
       </c>
       <c r="D10" t="s">
-        <v>208</v>
+        <v>414</v>
       </c>
       <c r="E10" t="s">
-        <v>209</v>
+        <v>415</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>186</v>
+        <v>416</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>210</v>
+        <v>417</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>211</v>
+        <v>418</v>
       </c>
       <c r="D11" t="s">
-        <v>208</v>
+        <v>419</v>
       </c>
       <c r="E11" t="s">
-        <v>212</v>
+        <v>420</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>190</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>213</v>
+        <v>422</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>214</v>
+        <v>423</v>
       </c>
       <c r="D12" t="s">
-        <v>215</v>
+        <v>424</v>
       </c>
       <c r="E12" t="s">
-        <v>216</v>
+        <v>425</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>195</v>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>428</v>
+      </c>
+      <c r="D13" t="s">
+        <v>429</v>
+      </c>
+      <c r="E13" t="s">
+        <v>430</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" t="s">
+        <v>433</v>
+      </c>
+      <c r="D14" t="s">
+        <v>434</v>
+      </c>
+      <c r="E14" t="s">
+        <v>435</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" t="s">
+        <v>438</v>
+      </c>
+      <c r="D15" t="s">
+        <v>439</v>
+      </c>
+      <c r="E15" t="s">
+        <v>440</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" t="s">
+        <v>443</v>
+      </c>
+      <c r="D16" t="s">
+        <v>444</v>
+      </c>
+      <c r="E16" t="s">
+        <v>445</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" t="s">
+        <v>447</v>
+      </c>
+      <c r="D17" t="s">
+        <v>444</v>
+      </c>
+      <c r="E17" t="s">
+        <v>448</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C18" t="s">
+        <v>450</v>
+      </c>
+      <c r="D18" t="s">
+        <v>451</v>
+      </c>
+      <c r="E18" t="s">
+        <v>452</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" t="s">
+        <v>454</v>
+      </c>
+      <c r="D19" t="s">
+        <v>455</v>
+      </c>
+      <c r="E19" t="s">
+        <v>456</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C20" t="s">
+        <v>459</v>
+      </c>
+      <c r="D20" t="s">
+        <v>460</v>
+      </c>
+      <c r="E20" t="s">
+        <v>461</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" t="s">
+        <v>464</v>
+      </c>
+      <c r="D21" t="s">
+        <v>465</v>
+      </c>
+      <c r="E21" t="s">
+        <v>466</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" t="s">
+        <v>469</v>
+      </c>
+      <c r="D22" t="s">
+        <v>470</v>
+      </c>
+      <c r="E22" t="s">
+        <v>471</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C23" t="s">
+        <v>474</v>
+      </c>
+      <c r="D23" t="s">
+        <v>475</v>
+      </c>
+      <c r="E23" t="s">
+        <v>476</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" t="s">
+        <v>479</v>
+      </c>
+      <c r="D24" t="s">
+        <v>475</v>
+      </c>
+      <c r="E24" t="s">
+        <v>480</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>483</v>
+      </c>
+      <c r="D25" t="s">
+        <v>484</v>
+      </c>
+      <c r="E25" t="s">
+        <v>485</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G25" t="s">
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -2596,506 +4719,506 @@
   <sheetData>
     <row r="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>217</v>
+        <v>487</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>218</v>
+        <v>488</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>219</v>
+        <v>489</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>220</v>
+        <v>490</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>221</v>
+        <v>491</v>
       </c>
       <c r="B2" t="s">
-        <v>222</v>
+        <v>492</v>
       </c>
       <c r="C2" t="s">
-        <v>223</v>
+        <v>493</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>224</v>
+        <v>494</v>
       </c>
       <c r="B3" t="s">
-        <v>225</v>
+        <v>495</v>
       </c>
       <c r="C3" t="s">
-        <v>226</v>
+        <v>496</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>227</v>
+        <v>497</v>
       </c>
       <c r="B4" t="s">
-        <v>228</v>
+        <v>498</v>
       </c>
       <c r="C4" t="s">
-        <v>229</v>
+        <v>499</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>230</v>
+        <v>500</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>501</v>
       </c>
       <c r="C5" t="s">
-        <v>232</v>
+        <v>502</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>233</v>
+        <v>503</v>
       </c>
       <c r="B6" t="s">
-        <v>234</v>
+        <v>504</v>
       </c>
       <c r="C6" t="s">
-        <v>235</v>
+        <v>505</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>236</v>
+        <v>506</v>
       </c>
       <c r="B7" t="s">
-        <v>237</v>
+        <v>507</v>
       </c>
       <c r="C7" t="s">
-        <v>238</v>
+        <v>508</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>239</v>
+        <v>509</v>
       </c>
       <c r="B8" t="s">
-        <v>240</v>
+        <v>510</v>
       </c>
       <c r="C8" t="s">
-        <v>241</v>
+        <v>511</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>242</v>
+        <v>512</v>
       </c>
       <c r="B9" t="s">
-        <v>243</v>
+        <v>513</v>
       </c>
       <c r="C9" t="s">
-        <v>244</v>
+        <v>514</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>245</v>
+        <v>515</v>
       </c>
       <c r="B10" t="s">
-        <v>246</v>
+        <v>516</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>517</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>248</v>
+        <v>518</v>
       </c>
       <c r="B11" t="s">
-        <v>249</v>
+        <v>519</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>520</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>251</v>
+        <v>521</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>522</v>
       </c>
       <c r="C12" t="s">
-        <v>253</v>
+        <v>523</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>254</v>
+        <v>524</v>
       </c>
       <c r="B13" t="s">
-        <v>255</v>
+        <v>525</v>
       </c>
       <c r="C13" t="s">
-        <v>256</v>
+        <v>526</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>257</v>
+        <v>527</v>
       </c>
       <c r="B14" t="s">
-        <v>258</v>
+        <v>528</v>
       </c>
       <c r="C14" t="s">
-        <v>259</v>
+        <v>529</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>260</v>
+        <v>530</v>
       </c>
       <c r="B15" t="s">
-        <v>261</v>
+        <v>531</v>
       </c>
       <c r="C15" t="s">
-        <v>262</v>
+        <v>532</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>263</v>
+        <v>533</v>
       </c>
       <c r="B16" t="s">
-        <v>264</v>
+        <v>534</v>
       </c>
       <c r="C16" t="s">
-        <v>265</v>
+        <v>535</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>266</v>
+        <v>536</v>
       </c>
       <c r="B17" t="s">
-        <v>267</v>
+        <v>537</v>
       </c>
       <c r="C17" t="s">
-        <v>268</v>
+        <v>538</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>269</v>
+        <v>539</v>
       </c>
       <c r="B18" t="s">
-        <v>270</v>
+        <v>540</v>
       </c>
       <c r="C18" t="s">
-        <v>271</v>
+        <v>541</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>272</v>
+        <v>542</v>
       </c>
       <c r="B19" t="s">
-        <v>273</v>
+        <v>543</v>
       </c>
       <c r="C19" t="s">
-        <v>271</v>
+        <v>541</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>274</v>
+        <v>544</v>
       </c>
       <c r="B20" t="s">
-        <v>275</v>
+        <v>545</v>
       </c>
       <c r="C20" t="s">
-        <v>276</v>
+        <v>546</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>277</v>
+        <v>547</v>
       </c>
       <c r="B21" t="s">
-        <v>278</v>
+        <v>548</v>
       </c>
       <c r="C21" t="s">
-        <v>279</v>
+        <v>549</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>280</v>
+        <v>550</v>
       </c>
       <c r="B22" t="s">
-        <v>281</v>
+        <v>551</v>
       </c>
       <c r="C22" t="s">
-        <v>282</v>
+        <v>552</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>283</v>
+        <v>553</v>
       </c>
       <c r="B23" t="s">
-        <v>284</v>
+        <v>554</v>
       </c>
       <c r="C23" t="s">
-        <v>285</v>
+        <v>555</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>286</v>
+        <v>556</v>
       </c>
       <c r="B24" t="s">
-        <v>287</v>
+        <v>557</v>
       </c>
       <c r="C24" t="s">
-        <v>288</v>
+        <v>558</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>289</v>
+        <v>559</v>
       </c>
       <c r="B25" t="s">
-        <v>290</v>
+        <v>560</v>
       </c>
       <c r="C25" t="s">
-        <v>291</v>
+        <v>561</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>292</v>
+        <v>562</v>
       </c>
       <c r="B26" t="s">
-        <v>293</v>
+        <v>563</v>
       </c>
       <c r="C26" t="s">
-        <v>294</v>
+        <v>564</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>295</v>
+        <v>565</v>
       </c>
       <c r="B27" t="s">
-        <v>296</v>
+        <v>566</v>
       </c>
       <c r="C27" t="s">
-        <v>297</v>
+        <v>567</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>298</v>
+        <v>568</v>
       </c>
       <c r="B28" t="s">
-        <v>299</v>
+        <v>569</v>
       </c>
       <c r="C28" t="s">
-        <v>300</v>
+        <v>570</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>301</v>
+        <v>571</v>
       </c>
       <c r="B29" t="s">
-        <v>302</v>
+        <v>572</v>
       </c>
       <c r="C29" t="s">
-        <v>303</v>
+        <v>573</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>304</v>
+        <v>574</v>
       </c>
       <c r="B30" t="s">
-        <v>305</v>
+        <v>575</v>
       </c>
       <c r="C30" t="s">
-        <v>306</v>
+        <v>576</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>307</v>
+        <v>577</v>
       </c>
       <c r="B31" t="s">
-        <v>308</v>
+        <v>578</v>
       </c>
       <c r="C31" t="s">
-        <v>309</v>
+        <v>579</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>310</v>
+        <v>580</v>
       </c>
       <c r="B32" t="s">
-        <v>311</v>
+        <v>581</v>
       </c>
       <c r="C32" t="s">
-        <v>312</v>
+        <v>582</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>313</v>
+        <v>583</v>
       </c>
       <c r="B33" t="s">
-        <v>314</v>
+        <v>584</v>
       </c>
       <c r="C33" t="s">
-        <v>315</v>
+        <v>585</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>316</v>
+        <v>586</v>
       </c>
       <c r="B34" t="s">
-        <v>317</v>
+        <v>587</v>
       </c>
       <c r="C34" t="s">
-        <v>318</v>
+        <v>588</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>319</v>
+        <v>589</v>
       </c>
       <c r="B35" t="s">
-        <v>320</v>
+        <v>590</v>
       </c>
       <c r="C35" t="s">
-        <v>321</v>
+        <v>591</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>322</v>
+        <v>592</v>
       </c>
       <c r="B36" t="s">
-        <v>323</v>
+        <v>593</v>
       </c>
       <c r="C36" t="s">
-        <v>324</v>
+        <v>594</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>